<commit_message>
fix equation name + refactoring
</commit_message>
<xml_diff>
--- a/omf-example-plugin/src/main/java/com/samares_engineering/omf/omf_example_plugin/features/excel_to_parametric/UAV MOE Equation.xlsx
+++ b/omf-example-plugin/src/main/java/com/samares_engineering/omf/omf_example_plugin/features/excel_to_parametric/UAV MOE Equation.xlsx
@@ -5,13 +5,15 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\workspace\java\mdplugins\OMF\OMF_Private\omf-example-plugin\src\main\java\com\samares_engineering\omf\omf_example_plugin\features\excel_to_parametric\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Workspace\Plugins\OMF_Private\omf-example-plugin\src\main\java\com\samares_engineering\omf\omf_example_plugin\features\excel_to_parametric\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB2AE45D-B832-477E-BAAF-ABFB79919A86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C49536D0-5DE2-4B5D-A098-7DA6590E691B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14670" windowHeight="10545" xr2:uid="{A22A8A54-8611-4DA6-995F-F1DD76DD8434}"/>
-    <workbookView xWindow="-105" yWindow="10440" windowWidth="14670" windowHeight="10545" activeTab="1" xr2:uid="{ECDD6195-D704-4DB1-91AF-46E52C29149A}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{A22A8A54-8611-4DA6-995F-F1DD76DD8434}"/>
+    <workbookView xWindow="-22308" yWindow="9144" windowWidth="17280" windowHeight="3240" xr2:uid="{ECDD6195-D704-4DB1-91AF-46E52C29149A}"/>
+    <workbookView xWindow="-11616" yWindow="8412" windowWidth="11712" windowHeight="13776" activeTab="1" xr2:uid="{798562BD-691F-4049-8B94-C5F37D32337C}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{5DB4170F-FB00-4D33-A0EA-EE7DB350FAE6}"/>
   </bookViews>
   <sheets>
     <sheet name="ValueProperties" sheetId="1" r:id="rId1"/>
@@ -787,17 +789,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81F39931-1C93-41B6-BB89-874B75E18699}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="32.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.5703125" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="32.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5546875" customWidth="1"/>
+    <col min="3" max="3" width="14.88671875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="37" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="88.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="88.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>5</v>
       </c>
@@ -808,7 +810,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>20</v>
       </c>
@@ -822,7 +824,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>21</v>
       </c>
@@ -836,7 +838,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>22</v>
       </c>
@@ -850,7 +852,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
         <v>23</v>
       </c>
@@ -864,7 +866,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>24</v>
       </c>
@@ -878,7 +880,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>19</v>
       </c>
@@ -892,7 +894,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>56</v>
       </c>
@@ -906,7 +908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>25</v>
       </c>
@@ -920,7 +922,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="12" t="s">
         <v>26</v>
       </c>
@@ -934,7 +936,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="13" t="s">
         <v>27</v>
       </c>
@@ -948,7 +950,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="14" t="s">
         <v>28</v>
       </c>
@@ -962,7 +964,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="15" t="s">
         <v>29</v>
       </c>
@@ -976,7 +978,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="16" t="s">
         <v>30</v>
       </c>
@@ -987,10 +989,10 @@
         <v>5</v>
       </c>
       <c r="D14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>31</v>
       </c>
@@ -1004,7 +1006,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>32</v>
       </c>
@@ -1026,15 +1028,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DA56FD2-2E8C-4F98-9B5F-251C6FDF40B3}">
   <dimension ref="A1:F17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="37.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="3" max="3" width="13.42578125" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="13.44140625" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>5</v>
       </c>
@@ -1051,7 +1053,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>33</v>
       </c>
@@ -1073,7 +1075,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>35</v>
       </c>
@@ -1091,7 +1093,7 @@
       </c>
       <c r="F3" s="1"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>34</v>
       </c>
@@ -1110,7 +1112,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>58</v>
       </c>
@@ -1129,7 +1131,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" ht="18" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
         <v>59</v>
       </c>
@@ -1151,7 +1153,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="18" x14ac:dyDescent="0.35">
       <c r="A7" s="12" t="s">
         <v>36</v>
       </c>
@@ -1169,7 +1171,7 @@
       </c>
       <c r="F7" s="2"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
         <v>37</v>
       </c>
@@ -1191,7 +1193,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" ht="18" x14ac:dyDescent="0.35">
       <c r="A9" s="13" t="s">
         <v>38</v>
       </c>
@@ -1213,7 +1215,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="22" t="s">
         <v>65</v>
       </c>
@@ -1228,7 +1230,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
         <v>63</v>
       </c>
@@ -1247,7 +1249,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="22" t="s">
         <v>39</v>
       </c>
@@ -1269,7 +1271,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="22" t="s">
         <v>40</v>
       </c>
@@ -1286,7 +1288,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
         <v>41</v>
       </c>
@@ -1308,7 +1310,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" ht="18" x14ac:dyDescent="0.35">
       <c r="A15" s="15" t="s">
         <v>42</v>
       </c>
@@ -1330,7 +1332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="16" t="s">
         <v>43</v>
       </c>
@@ -1352,7 +1354,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:6" s="26" customFormat="1" ht="21" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" s="26" customFormat="1" ht="21" x14ac:dyDescent="0.4">
       <c r="A17" s="23" t="s">
         <v>43</v>
       </c>

</xml_diff>